<commit_message>
Add form submission and output generation workflow
</commit_message>
<xml_diff>
--- a/Config/Config.xlsx
+++ b/Config/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Test\DemoQa_Form_Automation\Config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DECFFB2-EB15-4B0F-AC10-48E5404BC695}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27ACD4CA-A191-4BD5-987E-0E4D5B240238}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7695" yWindow="3900" windowWidth="14400" windowHeight="8205" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>Key</t>
   </si>
@@ -69,6 +69,9 @@
   </si>
   <si>
     <t>Data</t>
+  </si>
+  <si>
+    <t>OutputTemplateFilePath</t>
   </si>
 </sst>
 </file>
@@ -429,7 +432,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.140625" customWidth="1"/>
@@ -485,6 +488,15 @@
         <v>10</v>
       </c>
     </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" t="str">
+        <f>_xlfn.CONCAT(B4,"DemoQA_Output_Template.xlsx")</f>
+        <v>Data\Output\DemoQA_Output_Template.xlsx</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" xr:uid="{07F4A3B6-2072-493B-B518-3EA6E30AFD60}"/>

</xml_diff>

<commit_message>
Resolve browser automation and submission issues
</commit_message>
<xml_diff>
--- a/Config/Config.xlsx
+++ b/Config/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Test\DemoQa_Form_Automation\Config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27ACD4CA-A191-4BD5-987E-0E4D5B240238}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5607354-BC07-40BA-A426-7E6C48F85C0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="7695" yWindow="3900" windowWidth="14400" windowHeight="8205" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,9 +38,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
-    <t>Key</t>
-  </si>
-  <si>
     <t>Value</t>
   </si>
   <si>
@@ -72,6 +69,9 @@
   </si>
   <si>
     <t>OutputTemplateFilePath</t>
+  </si>
+  <si>
+    <t>Name</t>
   </si>
 </sst>
 </file>
@@ -441,39 +441,39 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B5" t="str">
         <f>_xlfn.CONCAT(B3,"DemoQA_Input.xlsx")</f>
@@ -482,15 +482,15 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" t="s">
         <v>9</v>
-      </c>
-      <c r="B6" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B7" t="str">
         <f>_xlfn.CONCAT(B4,"DemoQA_Output_Template.xlsx")</f>

</xml_diff>

<commit_message>
Enhance input validation and retry handling
</commit_message>
<xml_diff>
--- a/Config/Config.xlsx
+++ b/Config/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Test\DemoQa_Form_Automation\Config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5607354-BC07-40BA-A426-7E6C48F85C0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A7CA82B-3B84-4B03-8112-4AB3E8B41775}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7695" yWindow="3900" windowWidth="14400" windowHeight="8205" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Implement output reporting, exception handling, and error screenshots
</commit_message>
<xml_diff>
--- a/Config/Config.xlsx
+++ b/Config/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Test\DemoQa_Form_Automation\Config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A7CA82B-3B84-4B03-8112-4AB3E8B41775}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B788F830-B251-4366-BC90-6784EB49C684}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>Value</t>
   </si>
@@ -72,6 +72,27 @@
   </si>
   <si>
     <t>Name</t>
+  </si>
+  <si>
+    <t>ScreenshotsFolderPath</t>
+  </si>
+  <si>
+    <t>Data\Screenshots\</t>
+  </si>
+  <si>
+    <t>OutputSheetName</t>
+  </si>
+  <si>
+    <t>Result</t>
+  </si>
+  <si>
+    <t>RetryCountAttempts</t>
+  </si>
+  <si>
+    <t>TemplateFolderPath</t>
+  </si>
+  <si>
+    <t>Data\Template\</t>
   </si>
 </sst>
 </file>
@@ -432,7 +453,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.140625" customWidth="1"/>
@@ -490,11 +511,43 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>10</v>
       </c>
-      <c r="B7" t="str">
-        <f>_xlfn.CONCAT(B4,"DemoQA_Output_Template.xlsx")</f>
-        <v>Data\Output\DemoQA_Output_Template.xlsx</v>
+      <c r="B8" t="str">
+        <f>_xlfn.CONCAT(B7,"DemoQA_Output_Template.xlsx")</f>
+        <v>Data\Template\DemoQA_Output_Template.xlsx</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Enhance configuration management and project documentation
</commit_message>
<xml_diff>
--- a/Config/Config.xlsx
+++ b/Config/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Test\DemoQa_Form_Automation\Config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B788F830-B251-4366-BC90-6784EB49C684}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{354980BC-13B7-44DE-96B6-645FFB3B44DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>Value</t>
   </si>
@@ -93,6 +93,12 @@
   </si>
   <si>
     <t>Data\Template\</t>
+  </si>
+  <si>
+    <t>OutputFileName</t>
+  </si>
+  <si>
+    <t>DemoQA_Output_{DateTime}.xlsx</t>
   </si>
 </sst>
 </file>
@@ -453,7 +459,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.140625" customWidth="1"/>
@@ -528,25 +534,33 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="B9" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B10" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>16</v>
       </c>
-      <c r="B11">
+      <c r="B12">
         <v>3</v>
       </c>
     </row>

</xml_diff>